<commit_message>
OCCF update to output 1000KRW
</commit_message>
<xml_diff>
--- a/InputData/web-app/OCCF/Output Currency Conversion Factors.xlsx
+++ b/InputData/web-app/OCCF/Output Currency Conversion Factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-southkorea\InputData\web-app\OCCF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\web-app\OCCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA38807-15E2-4E49-8980-288C6A38AA58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8360B5E7-EDDC-4730-8C2D-9AF82BA8A78E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="OCCF-DpMOCU" sheetId="4" r:id="rId3"/>
     <sheet name="OCCF-DpSOCU" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" iterateDelta="1.0000000000000001E-5"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
   <si>
     <t>Source:</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>2019 dollars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">units are in 1000 KWR </t>
   </si>
 </sst>
 </file>
@@ -188,17 +191,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
@@ -220,9 +221,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -260,9 +261,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -295,26 +296,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -347,26 +331,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -540,29 +507,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C38"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" customWidth="1"/>
-    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.453125" customWidth="1"/>
+    <col min="2" max="2" width="26.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -570,80 +537,80 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="6"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="5"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="6"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="6"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B23" s="5"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>0.89805481563188172</v>
       </c>
@@ -651,50 +618,55 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B36">
         <v>1164.79</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="7" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -712,23 +684,23 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3">
-        <f>10^9*About!$A$26/About!$B$36</f>
-        <v>771001.48149613384</v>
+      <c r="B2" s="2">
+        <f>(10^9*About!$A$26/About!$B$36)*1000</f>
+        <v>771001481.4961338</v>
       </c>
     </row>
   </sheetData>
@@ -742,23 +714,23 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3">
-        <f>10^6*About!$A$26/About!$B$36</f>
-        <v>771.00148149613381</v>
+      <c r="B2" s="2">
+        <f>(10^6*About!$A$26/About!$B$36)*1000</f>
+        <v>771001.48149613384</v>
       </c>
     </row>
   </sheetData>
@@ -772,23 +744,23 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="7">
-        <f>About!A26/About!$B$36</f>
-        <v>7.7100148149613387E-4</v>
+      <c r="B2">
+        <f>(About!A26/About!$B$36)*1000</f>
+        <v>0.7710014814961339</v>
       </c>
     </row>
   </sheetData>
@@ -956,13 +928,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EE0DCE0-21BD-4BBD-B5BF-DB017A2506C3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EE0DCE0-21BD-4BBD-B5BF-DB017A2506C3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6EF2122-C1FB-4A3B-84B8-29D6F42C74CA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6EF2122-C1FB-4A3B-84B8-29D6F42C74CA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{704CAEF7-E5E9-4A87-B274-39F747162F2D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{704CAEF7-E5E9-4A87-B274-39F747162F2D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>